<commit_message>
Auto update Pengadaan 2026-10-13 08:09:05
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>674360508</v>
+        <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>134654115</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2261946920</v>
+        <v>2271451073</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1551,22 +1559,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>225945607</v>
+        <v>75945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1622,13 +1630,13 @@
         <v>127</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>801667671</v>
+        <v>805287130</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>103722907</v>
+        <v>107342366</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1789,25 +1797,25 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>618811959</v>
+        <v>903293859</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>177204602</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1094433360</v>
+        <v>451166160</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J37" s="11" t="n">
         <v>441607357</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -1996,13 +2004,13 @@
         <v>41</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>458240143</v>
+        <v>438619561</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>54570486</v>
+        <v>34949904</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>83626512</v>
+        <v>72726534</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2347,24 +2355,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3320,13 +3334,13 @@
         <v>157</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1492823770</v>
+        <v>1495540870</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>27</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>219640414</v>
+        <v>222357514</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>27</v>
@@ -3349,25 +3363,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3934</v>
+        <v>3894</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32214390422</v>
+        <v>32523552181</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>469</v>
+        <v>430</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6513005593</v>
+        <v>6822167352</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>469</v>
+        <v>430</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>10273885518.6</v>
+        <v>6376034170.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>25701384829</v>
@@ -3791,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4592,28 +4606,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1346095756</v>
+        <v>1566751699</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1004886595</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4834,28 +4848,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5188,40 +5202,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>1831557010</v>
+        <v>2573425510</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>1283221951</v>
+        <v>1936290451</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1247082323</v>
+        <v>1890349523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>852976373</v>
+        <v>1496243573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>188207363</v>
+        <v>313637363</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N37" s="11" t="n">
-        <v>548335059</v>
+        <v>637135059</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5570,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -6034,40 +6048,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7219,13 +7221,13 @@
         <v>4</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>467474077</v>
+        <v>498477099</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>115814581</v>
+        <v>146817603</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7534,40 +7536,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>816</v>
+        <v>832</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>96810977021</v>
+        <v>98382669008</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64297726774</v>
+        <v>65780618761</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63140628290.41</v>
+        <v>64056546862.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>293</v>
+        <v>308</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37013603546.02</v>
+        <v>37929522118.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>753913873</v>
+        <v>879343873</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>32513250247</v>
+        <v>32602050247</v>
       </c>
     </row>
   </sheetData>
@@ -8369,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26394591741</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24599146241</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>21</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24599146241</v>
+        <v>26394591741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8588,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8813,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12007,34 +12009,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>136252934738</v>
+        <v>180688297475</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>100827252631</v>
+        <v>145262615368</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>67290962337.01</v>
+        <v>70271840613.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>62842528537</v>
+        <v>65823406813</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2915140258</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-13 10:10:30
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1389,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>677290237</v>
+        <v>674360508</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>137583844</v>
+        <v>134654115</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1345382085</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1528,13 +1520,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2271451073</v>
+        <v>2261946920</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1559,22 +1551,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>75945607</v>
+        <v>225945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1630,13 +1622,13 @@
         <v>127</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>805287130</v>
+        <v>801667671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1797,25 +1789,25 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>903293859</v>
+        <v>618811959</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>461686502</v>
+        <v>177204602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>451166160</v>
+        <v>1094433360</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J37" s="11" t="n">
         <v>441607357</v>
@@ -1868,13 +1860,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1305525621</v>
+        <v>1279995621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>378058156</v>
+        <v>352528156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -2004,13 +1996,13 @@
         <v>41</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>438619561</v>
+        <v>458240143</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2035,22 +2027,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2355,30 +2347,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3334,13 +3320,13 @@
         <v>157</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1495540870</v>
+        <v>1492823770</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>27</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>222357514</v>
+        <v>219640414</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>27</v>
@@ -3363,25 +3349,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3894</v>
+        <v>3934</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32523552181</v>
+        <v>32214390422</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>430</v>
+        <v>469</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6822167352</v>
+        <v>6513005593</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>430</v>
+        <v>469</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6376034170.6</v>
+        <v>10273885518.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3464</v>
+        <v>3465</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>25701384829</v>
@@ -3805,13 +3791,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4606,28 +4592,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1566751699</v>
+        <v>1346095756</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1225542538</v>
+        <v>1004886595</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4848,28 +4834,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5202,40 +5188,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>2573425510</v>
+        <v>1831557010</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>1936290451</v>
+        <v>1283221951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1890349523</v>
+        <v>1247082323</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>1496243573</v>
+        <v>852976373</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>313637363</v>
+        <v>188207363</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N37" s="11" t="n">
-        <v>637135059</v>
+        <v>548335059</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5584,28 +5570,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>523391100</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -6048,28 +6034,40 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>660566066</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>340582172</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" s="9" t="n">
-        <v>68020787</v>
+        <v>319983894</v>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7221,13 +7219,13 @@
         <v>4</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>498477099</v>
+        <v>467474077</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7536,40 +7534,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>98382669008</v>
+        <v>96810977021</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>519</v>
+        <v>504</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>65780618761</v>
+        <v>64297726774</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>519</v>
+        <v>504</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64056546862.41</v>
+        <v>63140628290.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>308</v>
+        <v>293</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37929522118.02</v>
+        <v>37013603546.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>879343873</v>
+        <v>753913873</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>32602050247</v>
+        <v>32513250247</v>
       </c>
     </row>
   </sheetData>
@@ -8371,28 +8369,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26394591741</v>
+        <v>24598091741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26394591741</v>
+        <v>24598091741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8590,13 +8588,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8815,34 +8813,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12009,34 +12007,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>240</v>
+        <v>216</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>180688297475</v>
+        <v>136252934738</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>145262615368</v>
+        <v>100827252631</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>160</v>
+        <v>136</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>70271840613.01001</v>
+        <v>67289907837.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65823406813</v>
+        <v>62841474037</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2915140258</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-13 12:09:09
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-13).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1381,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>674360508</v>
+        <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>134654115</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1520,13 +1528,13 @@
         <v>172</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2261946920</v>
+        <v>2271451073</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1551,22 +1559,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>225945607</v>
+        <v>75945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1622,13 +1630,13 @@
         <v>127</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>801667671</v>
+        <v>805287130</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>103722907</v>
+        <v>107342366</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1789,25 +1797,25 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>618811959</v>
+        <v>903293859</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>177204602</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1094433360</v>
+        <v>451166160</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J37" s="11" t="n">
         <v>441607357</v>
@@ -1860,13 +1868,13 @@
         <v>112</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1279995621</v>
+        <v>1305525621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -1996,13 +2004,13 @@
         <v>41</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>458240143</v>
+        <v>438619561</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>54570486</v>
+        <v>34949904</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2027,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>83626512</v>
+        <v>72726534</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2347,24 +2355,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3320,13 +3334,13 @@
         <v>157</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1492823770</v>
+        <v>1495540870</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>27</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>219640414</v>
+        <v>222357514</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>27</v>
@@ -3349,25 +3363,25 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3934</v>
+        <v>3894</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32214390422</v>
+        <v>32523552181</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>469</v>
+        <v>430</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6513005593</v>
+        <v>6822167352</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>469</v>
+        <v>430</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>10273885518.6</v>
+        <v>6376034170.6</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>3465</v>
+        <v>3464</v>
       </c>
       <c r="J77" s="13" t="n">
         <v>25701384829</v>
@@ -3791,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4592,28 +4606,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1346095756</v>
+        <v>1566751699</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1004886595</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4834,28 +4848,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5188,40 +5202,40 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>1831557010</v>
+        <v>2573425510</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>1283221951</v>
+        <v>1936290451</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1247082323</v>
+        <v>1890349523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>852976373</v>
+        <v>1496243573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>188207363</v>
+        <v>313637363</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N37" s="11" t="n">
-        <v>548335059</v>
+        <v>637135059</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -5570,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -6034,40 +6048,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7219,13 +7221,13 @@
         <v>4</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>467474077</v>
+        <v>498477099</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>115814581</v>
+        <v>146817603</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7534,40 +7536,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>816</v>
+        <v>832</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>96810977021</v>
+        <v>98382669008</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>64297726774</v>
+        <v>65780618761</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63140628290.41</v>
+        <v>64056546862.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>293</v>
+        <v>308</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37013603546.02</v>
+        <v>37929522118.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>753913873</v>
+        <v>879343873</v>
       </c>
       <c r="M77" s="12" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>32513250247</v>
+        <v>32602050247</v>
       </c>
     </row>
   </sheetData>
@@ -8369,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26394591741</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24598091741</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>21</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24598091741</v>
+        <v>26394591741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8588,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8813,34 +8815,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -12007,34 +12009,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>216</v>
+        <v>240</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>136252934738</v>
+        <v>180688297475</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>100827252631</v>
+        <v>145262615368</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>67289907837.01</v>
+        <v>70271840613.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>62841474037</v>
+        <v>65823406813</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2915140258</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>80</v>

</xml_diff>